<commit_message>
feat: agregar AnalizarFacturas, extract_pdf y archivos pendientes
</commit_message>
<xml_diff>
--- a/plantillas/LISTA base.xlsx
+++ b/plantillas/LISTA base.xlsx
@@ -5,7 +5,7 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Usuario\Documents\Default Project\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Usuario\Documents\Default Project\plantillas\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -877,671 +877,42 @@
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>141511</xdr:colOff>
+      <xdr:colOff>190500</xdr:colOff>
       <xdr:row>0</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>6</xdr:col>
-      <xdr:colOff>123825</xdr:colOff>
+      <xdr:colOff>296994</xdr:colOff>
       <xdr:row>8</xdr:row>
-      <xdr:rowOff>132183</xdr:rowOff>
+      <xdr:rowOff>84667</xdr:rowOff>
     </xdr:to>
-    <xdr:grpSp>
-      <xdr:nvGrpSpPr>
-        <xdr:cNvPr id="2" name="Grupo 1"/>
-        <xdr:cNvGrpSpPr/>
-      </xdr:nvGrpSpPr>
-      <xdr:grpSpPr>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Imagen 1"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
         <a:xfrm>
-          <a:off x="395511" y="0"/>
-          <a:ext cx="6787397" cy="1751433"/>
-          <a:chOff x="398686" y="0"/>
-          <a:chExt cx="6954614" cy="1770483"/>
+          <a:off x="444500" y="0"/>
+          <a:ext cx="6922161" cy="1703917"/>
         </a:xfrm>
-      </xdr:grpSpPr>
-      <xdr:pic>
-        <xdr:nvPicPr>
-          <xdr:cNvPr id="12521" name="Imagen 2">
-            <a:extLst>
-              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-0000E9300000}"/>
-              </a:ext>
-            </a:extLst>
-          </xdr:cNvPr>
-          <xdr:cNvPicPr>
-            <a:picLocks noChangeAspect="1"/>
-          </xdr:cNvPicPr>
-        </xdr:nvPicPr>
-        <xdr:blipFill>
-          <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print">
-            <a:extLst>
-              <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-                <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-              </a:ext>
-            </a:extLst>
-          </a:blip>
-          <a:srcRect/>
-          <a:stretch>
-            <a:fillRect/>
-          </a:stretch>
-        </xdr:blipFill>
-        <xdr:spPr bwMode="auto">
-          <a:xfrm>
-            <a:off x="491010" y="821923"/>
-            <a:ext cx="1584973" cy="360333"/>
-          </a:xfrm>
-          <a:prstGeom prst="rect">
-            <a:avLst/>
-          </a:prstGeom>
-          <a:noFill/>
-          <a:ln>
-            <a:noFill/>
-          </a:ln>
-          <a:extLst>
-            <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
-              <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
-                <a:solidFill>
-                  <a:srgbClr val="FFFFFF"/>
-                </a:solidFill>
-              </a14:hiddenFill>
-            </a:ext>
-            <a:ext uri="{91240B29-F687-4F45-9708-019B960494DF}">
-              <a14:hiddenLine xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" w="9525">
-                <a:solidFill>
-                  <a:srgbClr val="000000"/>
-                </a:solidFill>
-                <a:miter lim="800000"/>
-                <a:headEnd/>
-                <a:tailEnd/>
-              </a14:hiddenLine>
-            </a:ext>
-          </a:extLst>
-        </xdr:spPr>
-      </xdr:pic>
-      <xdr:pic>
-        <xdr:nvPicPr>
-          <xdr:cNvPr id="12526" name="Imagen 17">
-            <a:extLst>
-              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-0000EE300000}"/>
-              </a:ext>
-            </a:extLst>
-          </xdr:cNvPr>
-          <xdr:cNvPicPr>
-            <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
-          </xdr:cNvPicPr>
-        </xdr:nvPicPr>
-        <xdr:blipFill>
-          <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2" cstate="print">
-            <a:extLst>
-              <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-                <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-              </a:ext>
-            </a:extLst>
-          </a:blip>
-          <a:srcRect/>
-          <a:stretch>
-            <a:fillRect/>
-          </a:stretch>
-        </xdr:blipFill>
-        <xdr:spPr bwMode="auto">
-          <a:xfrm>
-            <a:off x="424655" y="1332029"/>
-            <a:ext cx="1742536" cy="360800"/>
-          </a:xfrm>
-          <a:prstGeom prst="rect">
-            <a:avLst/>
-          </a:prstGeom>
-          <a:noFill/>
-          <a:ln>
-            <a:noFill/>
-          </a:ln>
-          <a:extLst>
-            <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
-              <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
-                <a:solidFill>
-                  <a:srgbClr val="FFFFFF"/>
-                </a:solidFill>
-              </a14:hiddenFill>
-            </a:ext>
-            <a:ext uri="{91240B29-F687-4F45-9708-019B960494DF}">
-              <a14:hiddenLine xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" w="9525">
-                <a:solidFill>
-                  <a:srgbClr val="000000"/>
-                </a:solidFill>
-                <a:miter lim="800000"/>
-                <a:headEnd/>
-                <a:tailEnd/>
-              </a14:hiddenLine>
-            </a:ext>
-          </a:extLst>
-        </xdr:spPr>
-      </xdr:pic>
-      <xdr:pic>
-        <xdr:nvPicPr>
-          <xdr:cNvPr id="12527" name="Imagen 18">
-            <a:extLst>
-              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-0000EF300000}"/>
-              </a:ext>
-            </a:extLst>
-          </xdr:cNvPr>
-          <xdr:cNvPicPr>
-            <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
-          </xdr:cNvPicPr>
-        </xdr:nvPicPr>
-        <xdr:blipFill>
-          <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3" cstate="print">
-            <a:extLst>
-              <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-                <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-              </a:ext>
-            </a:extLst>
-          </a:blip>
-          <a:srcRect/>
-          <a:stretch>
-            <a:fillRect/>
-          </a:stretch>
-        </xdr:blipFill>
-        <xdr:spPr bwMode="auto">
-          <a:xfrm>
-            <a:off x="3949894" y="1351968"/>
-            <a:ext cx="1470711" cy="418515"/>
-          </a:xfrm>
-          <a:prstGeom prst="rect">
-            <a:avLst/>
-          </a:prstGeom>
-          <a:noFill/>
-          <a:ln>
-            <a:noFill/>
-          </a:ln>
-          <a:extLst>
-            <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
-              <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
-                <a:solidFill>
-                  <a:srgbClr val="FFFFFF"/>
-                </a:solidFill>
-              </a14:hiddenFill>
-            </a:ext>
-            <a:ext uri="{91240B29-F687-4F45-9708-019B960494DF}">
-              <a14:hiddenLine xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" w="9525">
-                <a:solidFill>
-                  <a:srgbClr val="000000"/>
-                </a:solidFill>
-                <a:miter lim="800000"/>
-                <a:headEnd/>
-                <a:tailEnd/>
-              </a14:hiddenLine>
-            </a:ext>
-          </a:extLst>
-        </xdr:spPr>
-      </xdr:pic>
-      <xdr:pic>
-        <xdr:nvPicPr>
-          <xdr:cNvPr id="12528" name="Imagen 23">
-            <a:extLst>
-              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-0000F0300000}"/>
-              </a:ext>
-            </a:extLst>
-          </xdr:cNvPr>
-          <xdr:cNvPicPr>
-            <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
-          </xdr:cNvPicPr>
-        </xdr:nvPicPr>
-        <xdr:blipFill>
-          <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4">
-            <a:extLst>
-              <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-                <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-              </a:ext>
-            </a:extLst>
-          </a:blip>
-          <a:srcRect/>
-          <a:stretch>
-            <a:fillRect/>
-          </a:stretch>
-        </xdr:blipFill>
-        <xdr:spPr bwMode="auto">
-          <a:xfrm>
-            <a:off x="2253319" y="810339"/>
-            <a:ext cx="1591833" cy="392547"/>
-          </a:xfrm>
-          <a:prstGeom prst="rect">
-            <a:avLst/>
-          </a:prstGeom>
-          <a:noFill/>
-          <a:ln>
-            <a:noFill/>
-          </a:ln>
-          <a:extLst>
-            <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
-              <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
-                <a:solidFill>
-                  <a:srgbClr val="FFFFFF"/>
-                </a:solidFill>
-              </a14:hiddenFill>
-            </a:ext>
-            <a:ext uri="{91240B29-F687-4F45-9708-019B960494DF}">
-              <a14:hiddenLine xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" w="9525">
-                <a:solidFill>
-                  <a:srgbClr val="000000"/>
-                </a:solidFill>
-                <a:miter lim="800000"/>
-                <a:headEnd/>
-                <a:tailEnd/>
-              </a14:hiddenLine>
-            </a:ext>
-          </a:extLst>
-        </xdr:spPr>
-      </xdr:pic>
-      <xdr:pic>
-        <xdr:nvPicPr>
-          <xdr:cNvPr id="12520" name="Imagen 1">
-            <a:extLst>
-              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-0000E8300000}"/>
-              </a:ext>
-            </a:extLst>
-          </xdr:cNvPr>
-          <xdr:cNvPicPr>
-            <a:picLocks noChangeAspect="1"/>
-          </xdr:cNvPicPr>
-        </xdr:nvPicPr>
-        <xdr:blipFill>
-          <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId5" cstate="print">
-            <a:extLst>
-              <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-                <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-              </a:ext>
-            </a:extLst>
-          </a:blip>
-          <a:srcRect/>
-          <a:stretch>
-            <a:fillRect/>
-          </a:stretch>
-        </xdr:blipFill>
-        <xdr:spPr bwMode="auto">
-          <a:xfrm>
-            <a:off x="398686" y="0"/>
-            <a:ext cx="1785741" cy="671909"/>
-          </a:xfrm>
-          <a:prstGeom prst="rect">
-            <a:avLst/>
-          </a:prstGeom>
-          <a:noFill/>
-          <a:ln>
-            <a:noFill/>
-          </a:ln>
-          <a:extLst>
-            <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
-              <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
-                <a:solidFill>
-                  <a:srgbClr val="FFFFFF"/>
-                </a:solidFill>
-              </a14:hiddenFill>
-            </a:ext>
-            <a:ext uri="{91240B29-F687-4F45-9708-019B960494DF}">
-              <a14:hiddenLine xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" w="9525">
-                <a:solidFill>
-                  <a:srgbClr val="000000"/>
-                </a:solidFill>
-                <a:miter lim="800000"/>
-                <a:headEnd/>
-                <a:tailEnd/>
-              </a14:hiddenLine>
-            </a:ext>
-          </a:extLst>
-        </xdr:spPr>
-      </xdr:pic>
-      <xdr:pic>
-        <xdr:nvPicPr>
-          <xdr:cNvPr id="12523" name="Imagen 4">
-            <a:extLst>
-              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-0000EB300000}"/>
-              </a:ext>
-            </a:extLst>
-          </xdr:cNvPr>
-          <xdr:cNvPicPr>
-            <a:picLocks noChangeAspect="1"/>
-          </xdr:cNvPicPr>
-        </xdr:nvPicPr>
-        <xdr:blipFill rotWithShape="1">
-          <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId6" cstate="print">
-            <a:extLst>
-              <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-                <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-              </a:ext>
-            </a:extLst>
-          </a:blip>
-          <a:srcRect l="3328" r="6518"/>
-          <a:stretch/>
-        </xdr:blipFill>
-        <xdr:spPr bwMode="auto">
-          <a:xfrm>
-            <a:off x="2271325" y="54343"/>
-            <a:ext cx="1486572" cy="588530"/>
-          </a:xfrm>
-          <a:prstGeom prst="rect">
-            <a:avLst/>
-          </a:prstGeom>
-          <a:noFill/>
-          <a:ln>
-            <a:noFill/>
-          </a:ln>
-          <a:extLst>
-            <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
-              <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
-                <a:solidFill>
-                  <a:srgbClr val="FFFFFF"/>
-                </a:solidFill>
-              </a14:hiddenFill>
-            </a:ext>
-            <a:ext uri="{91240B29-F687-4F45-9708-019B960494DF}">
-              <a14:hiddenLine xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" w="9525">
-                <a:solidFill>
-                  <a:srgbClr val="000000"/>
-                </a:solidFill>
-                <a:miter lim="800000"/>
-                <a:headEnd/>
-                <a:tailEnd/>
-              </a14:hiddenLine>
-            </a:ext>
-          </a:extLst>
-        </xdr:spPr>
-      </xdr:pic>
-      <xdr:pic>
-        <xdr:nvPicPr>
-          <xdr:cNvPr id="12524" name="Imagen 5">
-            <a:extLst>
-              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-0000EC300000}"/>
-              </a:ext>
-            </a:extLst>
-          </xdr:cNvPr>
-          <xdr:cNvPicPr>
-            <a:picLocks noChangeAspect="1"/>
-          </xdr:cNvPicPr>
-        </xdr:nvPicPr>
-        <xdr:blipFill>
-          <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId7" cstate="print">
-            <a:extLst>
-              <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-                <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-              </a:ext>
-            </a:extLst>
-          </a:blip>
-          <a:srcRect l="19180" t="38872" r="18921" b="40109"/>
-          <a:stretch>
-            <a:fillRect/>
-          </a:stretch>
-        </xdr:blipFill>
-        <xdr:spPr bwMode="auto">
-          <a:xfrm>
-            <a:off x="5667797" y="56348"/>
-            <a:ext cx="1527271" cy="580976"/>
-          </a:xfrm>
-          <a:prstGeom prst="rect">
-            <a:avLst/>
-          </a:prstGeom>
-          <a:noFill/>
-          <a:ln>
-            <a:noFill/>
-          </a:ln>
-          <a:extLst>
-            <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
-              <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
-                <a:solidFill>
-                  <a:srgbClr val="FFFFFF"/>
-                </a:solidFill>
-              </a14:hiddenFill>
-            </a:ext>
-            <a:ext uri="{91240B29-F687-4F45-9708-019B960494DF}">
-              <a14:hiddenLine xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" w="9525">
-                <a:solidFill>
-                  <a:srgbClr val="000000"/>
-                </a:solidFill>
-                <a:miter lim="800000"/>
-                <a:headEnd/>
-                <a:tailEnd/>
-              </a14:hiddenLine>
-            </a:ext>
-          </a:extLst>
-        </xdr:spPr>
-      </xdr:pic>
-      <xdr:pic>
-        <xdr:nvPicPr>
-          <xdr:cNvPr id="15" name="Imagen 14" descr="https://seekvectorlogo.com/wp-content/uploads/2018/03/moog-vector-logo.png">
-            <a:extLst>
-              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-00000F000000}"/>
-              </a:ext>
-            </a:extLst>
-          </xdr:cNvPr>
-          <xdr:cNvPicPr>
-            <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
-          </xdr:cNvPicPr>
-        </xdr:nvPicPr>
-        <xdr:blipFill rotWithShape="1">
-          <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId8" cstate="print">
-            <a:extLst>
-              <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-                <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-              </a:ext>
-            </a:extLst>
-          </a:blip>
-          <a:srcRect l="1675" t="30078" r="1195" b="30368"/>
-          <a:stretch/>
-        </xdr:blipFill>
-        <xdr:spPr bwMode="auto">
-          <a:xfrm>
-            <a:off x="5672975" y="790622"/>
-            <a:ext cx="1499517" cy="395706"/>
-          </a:xfrm>
-          <a:prstGeom prst="rect">
-            <a:avLst/>
-          </a:prstGeom>
-          <a:noFill/>
-          <a:extLst>
-            <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
-              <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
-                <a:solidFill>
-                  <a:srgbClr val="FFFFFF"/>
-                </a:solidFill>
-              </a14:hiddenFill>
-            </a:ext>
-          </a:extLst>
-        </xdr:spPr>
-      </xdr:pic>
-      <xdr:pic>
-        <xdr:nvPicPr>
-          <xdr:cNvPr id="18" name="Imagen 17" descr="https://logos-download.com/wp-content/uploads/2018/05/Champion_logo_red.png">
-            <a:extLst>
-              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-000012000000}"/>
-              </a:ext>
-            </a:extLst>
-          </xdr:cNvPr>
-          <xdr:cNvPicPr>
-            <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
-          </xdr:cNvPicPr>
-        </xdr:nvPicPr>
-        <xdr:blipFill rotWithShape="1">
-          <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId9" cstate="print">
-            <a:extLst>
-              <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-                <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-              </a:ext>
-            </a:extLst>
-          </a:blip>
-          <a:srcRect l="3847" t="27178" r="3724" b="26934"/>
-          <a:stretch/>
-        </xdr:blipFill>
-        <xdr:spPr bwMode="auto">
-          <a:xfrm>
-            <a:off x="3854830" y="99769"/>
-            <a:ext cx="1675962" cy="500306"/>
-          </a:xfrm>
-          <a:prstGeom prst="rect">
-            <a:avLst/>
-          </a:prstGeom>
-          <a:noFill/>
-          <a:extLst>
-            <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
-              <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
-                <a:solidFill>
-                  <a:srgbClr val="FFFFFF"/>
-                </a:solidFill>
-              </a14:hiddenFill>
-            </a:ext>
-          </a:extLst>
-        </xdr:spPr>
-      </xdr:pic>
-      <xdr:pic>
-        <xdr:nvPicPr>
-          <xdr:cNvPr id="12" name="Imagen 11" descr="Fel-Pro Sealed Power 260-1016 Overhaul Gasket Kit 70-80 400 Small Block ..."/>
-          <xdr:cNvPicPr>
-            <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
-          </xdr:cNvPicPr>
-        </xdr:nvPicPr>
-        <xdr:blipFill>
-          <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId10" cstate="print">
-            <a:extLst>
-              <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-                <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-              </a:ext>
-            </a:extLst>
-          </a:blip>
-          <a:srcRect/>
-          <a:stretch>
-            <a:fillRect/>
-          </a:stretch>
-        </xdr:blipFill>
-        <xdr:spPr bwMode="auto">
-          <a:xfrm>
-            <a:off x="5562601" y="1338948"/>
-            <a:ext cx="1790699" cy="325641"/>
-          </a:xfrm>
-          <a:prstGeom prst="rect">
-            <a:avLst/>
-          </a:prstGeom>
-          <a:noFill/>
-          <a:extLst>
-            <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
-              <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
-                <a:solidFill>
-                  <a:srgbClr val="FFFFFF"/>
-                </a:solidFill>
-              </a14:hiddenFill>
-            </a:ext>
-          </a:extLst>
-        </xdr:spPr>
-      </xdr:pic>
-      <xdr:pic>
-        <xdr:nvPicPr>
-          <xdr:cNvPr id="13" name="Imagen 12" descr="Moresa Logo Vector - (.Ai .PNG .SVG .EPS Free Download)"/>
-          <xdr:cNvPicPr>
-            <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
-          </xdr:cNvPicPr>
-        </xdr:nvPicPr>
-        <xdr:blipFill>
-          <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId11" cstate="print">
-            <a:extLst>
-              <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-                <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-              </a:ext>
-            </a:extLst>
-          </a:blip>
-          <a:srcRect/>
-          <a:stretch>
-            <a:fillRect/>
-          </a:stretch>
-        </xdr:blipFill>
-        <xdr:spPr bwMode="auto">
-          <a:xfrm>
-            <a:off x="2295525" y="1078738"/>
-            <a:ext cx="1577321" cy="607187"/>
-          </a:xfrm>
-          <a:prstGeom prst="rect">
-            <a:avLst/>
-          </a:prstGeom>
-          <a:noFill/>
-          <a:extLst>
-            <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
-              <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
-                <a:solidFill>
-                  <a:srgbClr val="FFFFFF"/>
-                </a:solidFill>
-              </a14:hiddenFill>
-            </a:ext>
-          </a:extLst>
-        </xdr:spPr>
-      </xdr:pic>
-      <xdr:pic>
-        <xdr:nvPicPr>
-          <xdr:cNvPr id="17" name="Imagen 16" descr="https://dacomsa.com/dacomsastorefront/medias/LOGO-TF-VICTOR-NORMAL-2-.jpg?context=bWFzdGVyfGltYWdlc3w4NTA2MnxpbWFnZS9qcGVnfGFHWmlMMmhqWmk4NE9ERXdPREEyTlRBNU5UazRMMHhQUjA4Z1ZFWWdWa2xEVkU5U0lFNVBVazFCVENBb01pa3VhbkJufGMzNmMwODgwZTI3YTdhZDBjNjA3YmQ4YTM1MzJjNmRkNTAwZThkMDM3MDU3NzRmYzcxODBhNGYxYjk2NDQzZDk"/>
-          <xdr:cNvPicPr>
-            <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
-          </xdr:cNvPicPr>
-        </xdr:nvPicPr>
-        <xdr:blipFill rotWithShape="1">
-          <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId12" cstate="print">
-            <a:extLst>
-              <a:ext uri="{BEBA8EAE-BF5A-486C-A8C5-ECC9F3942E4B}">
-                <a14:imgProps xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
-                  <a14:imgLayer r:embed="rId13">
-                    <a14:imgEffect>
-                      <a14:backgroundRemoval t="25416" b="66271" l="1883" r="100000">
-                        <a14:foregroundMark x1="37029" y1="62708" x2="37029" y2="62708"/>
-                        <a14:foregroundMark x1="43724" y1="61995" x2="43724" y2="61995"/>
-                        <a14:foregroundMark x1="49163" y1="62708" x2="49163" y2="62708"/>
-                        <a14:foregroundMark x1="65690" y1="59145" x2="65690" y2="59145"/>
-                        <a14:foregroundMark x1="71757" y1="62708" x2="71757" y2="62708"/>
-                        <a14:foregroundMark x1="87238" y1="61995" x2="87238" y2="61995"/>
-                        <a14:foregroundMark x1="93933" y1="60570" x2="93933" y2="60570"/>
-                        <a14:foregroundMark x1="19247" y1="62708" x2="19247" y2="62708"/>
-                        <a14:foregroundMark x1="16736" y1="57957" x2="16736" y2="57957"/>
-                        <a14:foregroundMark x1="8159" y1="55107" x2="8159" y2="55107"/>
-                        <a14:foregroundMark x1="96862" y1="51544" x2="96862" y2="51544"/>
-                      </a14:backgroundRemoval>
-                    </a14:imgEffect>
-                  </a14:imgLayer>
-                </a14:imgProps>
-              </a:ext>
-              <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-                <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-              </a:ext>
-            </a:extLst>
-          </a:blip>
-          <a:srcRect t="20652" b="28262"/>
-          <a:stretch/>
-        </xdr:blipFill>
-        <xdr:spPr bwMode="auto">
-          <a:xfrm>
-            <a:off x="3987356" y="583877"/>
-            <a:ext cx="1537144" cy="646141"/>
-          </a:xfrm>
-          <a:prstGeom prst="rect">
-            <a:avLst/>
-          </a:prstGeom>
-          <a:noFill/>
-          <a:extLst>
-            <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
-              <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
-                <a:solidFill>
-                  <a:srgbClr val="FFFFFF"/>
-                </a:solidFill>
-              </a14:hiddenFill>
-            </a:ext>
-          </a:extLst>
-        </xdr:spPr>
-      </xdr:pic>
-    </xdr:grpSp>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
@@ -1839,9 +1210,9 @@
   <cols>
     <col min="1" max="1" width="3.85546875" customWidth="1"/>
     <col min="2" max="2" width="17" style="8" customWidth="1"/>
-    <col min="3" max="3" width="42.7109375" style="9" customWidth="1"/>
+    <col min="3" max="3" width="41.85546875" style="9" customWidth="1"/>
     <col min="4" max="4" width="16" style="15" customWidth="1"/>
-    <col min="5" max="5" width="15.42578125" style="15" customWidth="1"/>
+    <col min="5" max="5" width="16.28515625" style="15" customWidth="1"/>
     <col min="6" max="6" width="11" style="1" customWidth="1"/>
     <col min="7" max="7" width="6.42578125" style="18" customWidth="1"/>
     <col min="8" max="8" width="17.140625" bestFit="1" customWidth="1"/>

</xml_diff>